<commit_message>
Extend market intelligence analytics and update documentation
</commit_message>
<xml_diff>
--- a/outputs/Market_Business_Strategy_Intelligence.xlsx
+++ b/outputs/Market_Business_Strategy_Intelligence.xlsx
@@ -12,15 +12,17 @@
     <sheet name="Pricing_Analysis" sheetId="3" r:id="rId3"/>
     <sheet name="Product_Positioning" sheetId="4" r:id="rId4"/>
     <sheet name="Strategic_Recommendations" sheetId="5" r:id="rId5"/>
-    <sheet name="Source_Register" sheetId="6" r:id="rId6"/>
-    <sheet name="Assumptions_Provenance" sheetId="7" r:id="rId7"/>
+    <sheet name="Market_Growth_SEBI" sheetId="6" r:id="rId6"/>
+    <sheet name="TAM_SAM_SOM_Scenarios" sheetId="7" r:id="rId7"/>
+    <sheet name="Source_Register" sheetId="8" r:id="rId8"/>
+    <sheet name="Assumptions_Provenance" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="359">
   <si>
     <t>kpi_name</t>
   </si>
@@ -118,7 +120,7 @@
     <t>verified</t>
   </si>
   <si>
-    <t>2026-09-12</t>
+    <t>2026-09-24</t>
   </si>
   <si>
     <t>AVG(battery_capacity_kwh) across models</t>
@@ -397,6 +399,12 @@
     <t>top_speed_kmh</t>
   </si>
   <si>
+    <t>price_bucket</t>
+  </si>
+  <si>
+    <t>value_rank</t>
+  </si>
+  <si>
     <t>price_percentile</t>
   </si>
   <si>
@@ -418,6 +426,18 @@
     <t>price_premium_vs_market_pct</t>
   </si>
   <si>
+    <t>mid-market</t>
+  </si>
+  <si>
+    <t>unpriced</t>
+  </si>
+  <si>
+    <t>budget</t>
+  </si>
+  <si>
+    <t>premium</t>
+  </si>
+  <si>
     <t>below market average</t>
   </si>
   <si>
@@ -433,9 +453,6 @@
     <t>model_name</t>
   </si>
   <si>
-    <t>price_bucket</t>
-  </si>
-  <si>
     <t>range_bucket</t>
   </si>
   <si>
@@ -466,18 +483,6 @@
     <t>manufacturer_portfolio_share_pct</t>
   </si>
   <si>
-    <t>mid-market</t>
-  </si>
-  <si>
-    <t>unpriced</t>
-  </si>
-  <si>
-    <t>budget</t>
-  </si>
-  <si>
-    <t>premium</t>
-  </si>
-  <si>
     <t>short-range</t>
   </si>
   <si>
@@ -649,6 +654,144 @@
     <t>Indian Electric 2W Intelligence — Evidence-Based Strategy</t>
   </si>
   <si>
+    <t>fiscal_year</t>
+  </si>
+  <si>
+    <t>calendar_year_end</t>
+  </si>
+  <si>
+    <t>industry_e2w_units</t>
+  </si>
+  <si>
+    <t>data_classification</t>
+  </si>
+  <si>
+    <t>yoy_growth_pct</t>
+  </si>
+  <si>
+    <t>cagr_fy2021_fy2024_pct</t>
+  </si>
+  <si>
+    <t>provenance_status</t>
+  </si>
+  <si>
+    <t>coverage_note</t>
+  </si>
+  <si>
+    <t>FY2021</t>
+  </si>
+  <si>
+    <t>FY2022</t>
+  </si>
+  <si>
+    <t>FY2023</t>
+  </si>
+  <si>
+    <t>FY2024</t>
+  </si>
+  <si>
+    <t>OBSERVED - SEBI RHP 2024</t>
+  </si>
+  <si>
+    <t>Ola Electric Mobility Limited RHP (August 2024) - SEBI statutory filing</t>
+  </si>
+  <si>
+    <t>verified_primary_source</t>
+  </si>
+  <si>
+    <t>National India e2W total; state-level breakdown not available from this source</t>
+  </si>
+  <si>
+    <t>Indian Electric 2W Intelligence — SEBI-Verified Market Growth (FY2021-FY2024)</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>verified_fy2024_industry_units</t>
+  </si>
+  <si>
+    <t>verified_source</t>
+  </si>
+  <si>
+    <t>fy2025_growth_assumption_pct</t>
+  </si>
+  <si>
+    <t>tam_units</t>
+  </si>
+  <si>
+    <t>tam_revenue_inr_crore</t>
+  </si>
+  <si>
+    <t>geographic_concentration_pct</t>
+  </si>
+  <si>
+    <t>segment_concentration_pct</t>
+  </si>
+  <si>
+    <t>sam_units</t>
+  </si>
+  <si>
+    <t>sam_revenue_inr_crore</t>
+  </si>
+  <si>
+    <t>attainable_share_pct</t>
+  </si>
+  <si>
+    <t>som_units</t>
+  </si>
+  <si>
+    <t>som_revenue_inr_crore</t>
+  </si>
+  <si>
+    <t>avg_price_per_unit_inr</t>
+  </si>
+  <si>
+    <t>data_classification_tam</t>
+  </si>
+  <si>
+    <t>data_classification_sam</t>
+  </si>
+  <si>
+    <t>data_classification_som</t>
+  </si>
+  <si>
+    <t>methodology_version</t>
+  </si>
+  <si>
+    <t>Conservative Case</t>
+  </si>
+  <si>
+    <t>Base Case</t>
+  </si>
+  <si>
+    <t>Upside Case</t>
+  </si>
+  <si>
+    <t>Slower adoption: policy delays, subsidy uncertainty</t>
+  </si>
+  <si>
+    <t>Moderate growth; PM E-DRIVE scheme operational</t>
+  </si>
+  <si>
+    <t>Strong adoption: PM E-DRIVE full deployment, grid expansion</t>
+  </si>
+  <si>
+    <t>OBSERVED (FY24) + ASSUMPTION (growth)</t>
+  </si>
+  <si>
+    <t>ASSUMPTION</t>
+  </si>
+  <si>
+    <t>v1.0 - 2026-09-24</t>
+  </si>
+  <si>
+    <t>Indian Electric 2W Intelligence — TAM/SAM/SOM Sizing Framework (3 Scenarios)</t>
+  </si>
+  <si>
     <t>dataset_name</t>
   </si>
   <si>
@@ -706,6 +849,9 @@
     <t>policy_incentive_timeline.csv</t>
   </si>
   <si>
+    <t>sebi_verified_industry_totals.csv</t>
+  </si>
+  <si>
     <t>data/raw/vahan_e2w_registrations_monthly.csv</t>
   </si>
   <si>
@@ -724,6 +870,9 @@
     <t>data/raw/verified_product_catalog_2025_2026.csv</t>
   </si>
   <si>
+    <t>data/raw/sebi_verified_industry_totals.csv</t>
+  </si>
+  <si>
     <t>Legacy generator claim: Vahan 4.0</t>
   </si>
   <si>
@@ -742,6 +891,9 @@
     <t>Official OEM product pages/brochures/press releases</t>
   </si>
   <si>
+    <t>Ola Electric Mobility Limited SEBI Red Herring Prospectus (RHP) August 2024</t>
+  </si>
+  <si>
     <t>https://analytics.parivahan.gov.in/analytics/publicdashboard/vahan</t>
   </si>
   <si>
@@ -754,6 +906,9 @@
     <t>See source_url in each row</t>
   </si>
   <si>
+    <t>https://www.sebi.gov.in/filings/</t>
+  </si>
+  <si>
     <t>2026-09-07</t>
   </si>
   <si>
@@ -787,6 +942,9 @@
     <t>20 states/UTs</t>
   </si>
   <si>
+    <t>India national</t>
+  </si>
+  <si>
     <t>monthly state</t>
   </si>
   <si>
@@ -802,6 +960,9 @@
     <t>policy period</t>
   </si>
   <si>
+    <t>annual fiscal year</t>
+  </si>
+  <si>
     <t>derived</t>
   </si>
   <si>
@@ -832,9 +993,6 @@
     <t>source_transcription_pending_document</t>
   </si>
   <si>
-    <t>verified_primary_source</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -857,6 +1015,9 @@
   </si>
   <si>
     <t>30 source-linked rows across 5 manufacturers. Prices are location/date/offer-specific; blank values mean the cited source did not support that field.</t>
+  </si>
+  <si>
+    <t>4 fiscal years only (FY2021-FY2024); national totals only; no state-level breakdown; rounded to nearest 1000 as presented in prospectus</t>
   </si>
   <si>
     <t>Indian Electric 2W Intelligence — Data Provenance Inventory</t>
@@ -3939,7 +4100,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
@@ -3950,21 +4111,23 @@
     <col min="6" max="6" width="17.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="16.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="17.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="27.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="31.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="18.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="27.7109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="31.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="A1" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="3" t="s">
         <v>49</v>
       </c>
@@ -4010,8 +4173,14 @@
       <c r="O2" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="P2" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="1" t="s">
         <v>76</v>
       </c>
@@ -4036,29 +4205,35 @@
       <c r="H3" s="1">
         <v>40499.67</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J3" s="1">
+        <v>27</v>
+      </c>
+      <c r="K3" s="1">
         <v>0.39</v>
       </c>
-      <c r="J3" s="1">
+      <c r="L3" s="1">
         <v>2</v>
       </c>
-      <c r="K3" s="1">
+      <c r="M3" s="1">
         <v>21</v>
       </c>
-      <c r="L3" s="1">
+      <c r="N3" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M3" s="1">
+      <c r="O3" s="1">
         <v>126499</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O3" s="1">
+      <c r="P3" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q3" s="1">
         <v>-10.9</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:17">
       <c r="A4" s="1" t="s">
         <v>77</v>
       </c>
@@ -4083,29 +4258,35 @@
       <c r="H4" s="1">
         <v>43833</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J4" s="1">
+        <v>29</v>
+      </c>
+      <c r="K4" s="1">
         <v>0.64</v>
       </c>
-      <c r="J4" s="1">
+      <c r="L4" s="1">
         <v>3</v>
       </c>
-      <c r="K4" s="1">
+      <c r="M4" s="1">
         <v>13</v>
       </c>
-      <c r="L4" s="1">
+      <c r="N4" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M4" s="1">
+      <c r="O4" s="1">
         <v>126499</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O4" s="1">
+      <c r="P4" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q4" s="1">
         <v>-3.6</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:17">
       <c r="A5" s="1" t="s">
         <v>78</v>
       </c>
@@ -4118,26 +4299,32 @@
       <c r="E5" s="1">
         <v>157</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J5" s="1">
+        <v>31</v>
+      </c>
+      <c r="K5" s="1">
         <v>0</v>
       </c>
-      <c r="J5" s="1">
+      <c r="L5" s="1">
         <v>1</v>
       </c>
-      <c r="K5" s="1">
+      <c r="M5" s="1">
         <v>35</v>
       </c>
-      <c r="L5" s="1">
+      <c r="N5" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M5" s="1">
+      <c r="O5" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N5" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="P5" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="1" t="s">
         <v>79</v>
       </c>
@@ -4150,26 +4337,32 @@
       <c r="E6" s="1">
         <v>161</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J6" s="1">
+        <v>31</v>
+      </c>
+      <c r="K6" s="1">
         <v>0</v>
       </c>
-      <c r="J6" s="1">
+      <c r="L6" s="1">
         <v>1</v>
       </c>
-      <c r="K6" s="1">
+      <c r="M6" s="1">
         <v>35</v>
       </c>
-      <c r="L6" s="1">
+      <c r="N6" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M6" s="1">
+      <c r="O6" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
+      <c r="P6" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="1" t="s">
         <v>80</v>
       </c>
@@ -4182,26 +4375,32 @@
       <c r="E7" s="1">
         <v>126</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J7" s="1">
+        <v>31</v>
+      </c>
+      <c r="K7" s="1">
         <v>0</v>
       </c>
-      <c r="J7" s="1">
+      <c r="L7" s="1">
         <v>2</v>
       </c>
-      <c r="K7" s="1">
+      <c r="M7" s="1">
         <v>35</v>
       </c>
-      <c r="L7" s="1">
+      <c r="N7" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M7" s="1">
+      <c r="O7" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15">
+      <c r="P7" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="1" t="s">
         <v>81</v>
       </c>
@@ -4214,26 +4413,32 @@
       <c r="E8" s="1">
         <v>161</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J8" s="1">
+        <v>31</v>
+      </c>
+      <c r="K8" s="1">
         <v>0</v>
       </c>
-      <c r="J8" s="1">
+      <c r="L8" s="1">
         <v>2</v>
       </c>
-      <c r="K8" s="1">
+      <c r="M8" s="1">
         <v>35</v>
       </c>
-      <c r="L8" s="1">
+      <c r="N8" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M8" s="1">
+      <c r="O8" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
+      <c r="P8" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="1" t="s">
         <v>82</v>
       </c>
@@ -4255,29 +4460,35 @@
       <c r="H9" s="1">
         <v>37295.17</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J9" s="1">
+        <v>20</v>
+      </c>
+      <c r="K9" s="1">
         <v>0.21</v>
       </c>
-      <c r="J9" s="1">
+      <c r="L9" s="1">
         <v>1</v>
       </c>
-      <c r="K9" s="1">
+      <c r="M9" s="1">
         <v>27</v>
       </c>
-      <c r="L9" s="1">
+      <c r="N9" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M9" s="1">
+      <c r="O9" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O9" s="1">
+      <c r="P9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q9" s="1">
         <v>-20.7</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:17">
       <c r="A10" s="1" t="s">
         <v>83</v>
       </c>
@@ -4299,29 +4510,35 @@
       <c r="H10" s="1">
         <v>37039.73</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J10" s="1">
+        <v>18</v>
+      </c>
+      <c r="K10" s="1">
         <v>0.73</v>
       </c>
-      <c r="J10" s="1">
+      <c r="L10" s="1">
         <v>3</v>
       </c>
-      <c r="K10" s="1">
+      <c r="M10" s="1">
         <v>10</v>
       </c>
-      <c r="L10" s="1">
+      <c r="N10" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M10" s="1">
+      <c r="O10" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N10" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O10" s="1">
+      <c r="P10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q10" s="1">
         <v>0.5</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:17">
       <c r="A11" s="1" t="s">
         <v>84</v>
       </c>
@@ -4343,29 +4560,35 @@
       <c r="H11" s="1">
         <v>44708.97</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J11" s="1">
+        <v>26</v>
+      </c>
+      <c r="K11" s="1">
         <v>0.55</v>
       </c>
-      <c r="J11" s="1">
+      <c r="L11" s="1">
         <v>3</v>
       </c>
-      <c r="K11" s="1">
+      <c r="M11" s="1">
         <v>16</v>
       </c>
-      <c r="L11" s="1">
+      <c r="N11" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M11" s="1">
+      <c r="O11" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O11" s="1">
+      <c r="P11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q11" s="1">
         <v>-4.9</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:17">
       <c r="A12" s="1" t="s">
         <v>85</v>
       </c>
@@ -4387,29 +4610,35 @@
       <c r="H12" s="1">
         <v>40445.14</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J12" s="1">
+        <v>25</v>
+      </c>
+      <c r="K12" s="1">
         <v>0.85</v>
       </c>
-      <c r="J12" s="1">
+      <c r="L12" s="1">
         <v>4</v>
       </c>
-      <c r="K12" s="1">
+      <c r="M12" s="1">
         <v>6</v>
       </c>
-      <c r="L12" s="1">
+      <c r="N12" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M12" s="1">
+      <c r="O12" s="1">
         <v>131126.5</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O12" s="1">
+      <c r="P12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q12" s="1">
         <v>9.800000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:17">
       <c r="A13" s="1" t="s">
         <v>86</v>
       </c>
@@ -4434,29 +4663,35 @@
       <c r="H13" s="1">
         <v>39419.06</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J13" s="1">
+        <v>24</v>
+      </c>
+      <c r="K13" s="1">
         <v>0.48</v>
       </c>
-      <c r="J13" s="1">
+      <c r="L13" s="1">
         <v>2</v>
       </c>
-      <c r="K13" s="1">
+      <c r="M13" s="1">
         <v>18</v>
       </c>
-      <c r="L13" s="1">
+      <c r="N13" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M13" s="1">
+      <c r="O13" s="1">
         <v>118070</v>
       </c>
-      <c r="N13" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O13" s="1">
+      <c r="P13" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q13" s="1">
         <v>-7.5</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:17">
       <c r="A14" s="1" t="s">
         <v>87</v>
       </c>
@@ -4481,29 +4716,35 @@
       <c r="H14" s="1">
         <v>36666.33</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J14" s="1">
+        <v>14</v>
+      </c>
+      <c r="K14" s="1">
         <v>0.24</v>
       </c>
-      <c r="J14" s="1">
+      <c r="L14" s="1">
         <v>1</v>
       </c>
-      <c r="K14" s="1">
+      <c r="M14" s="1">
         <v>26</v>
       </c>
-      <c r="L14" s="1">
+      <c r="N14" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M14" s="1">
+      <c r="O14" s="1">
         <v>118070</v>
       </c>
-      <c r="N14" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O14" s="1">
+      <c r="P14" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q14" s="1">
         <v>-19.3</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:17">
       <c r="A15" s="1" t="s">
         <v>88</v>
       </c>
@@ -4519,26 +4760,32 @@
       <c r="F15" s="1">
         <v>63</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J15" s="1">
+        <v>31</v>
+      </c>
+      <c r="K15" s="1">
         <v>0</v>
       </c>
-      <c r="J15" s="1">
+      <c r="L15" s="1">
         <v>3</v>
       </c>
-      <c r="K15" s="1">
+      <c r="M15" s="1">
         <v>35</v>
       </c>
-      <c r="L15" s="1">
+      <c r="N15" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M15" s="1">
+      <c r="O15" s="1">
         <v>116168</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15">
+      <c r="P15" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="1" t="s">
         <v>89</v>
       </c>
@@ -4563,29 +4810,35 @@
       <c r="H16" s="1">
         <v>38428.57</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J16" s="1">
+        <v>19</v>
+      </c>
+      <c r="K16" s="1">
         <v>0.67</v>
       </c>
-      <c r="J16" s="1">
+      <c r="L16" s="1">
         <v>3</v>
       </c>
-      <c r="K16" s="1">
+      <c r="M16" s="1">
         <v>12</v>
       </c>
-      <c r="L16" s="1">
+      <c r="N16" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M16" s="1">
+      <c r="O16" s="1">
         <v>116168</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O16" s="1">
+      <c r="P16" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q16" s="1">
         <v>-1.4</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:17">
       <c r="A17" s="1" t="s">
         <v>90</v>
       </c>
@@ -4610,29 +4863,35 @@
       <c r="H17" s="1">
         <v>35000</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J17" s="1">
+        <v>12</v>
+      </c>
+      <c r="K17" s="1">
         <v>0.42</v>
       </c>
-      <c r="J17" s="1">
+      <c r="L17" s="1">
         <v>2</v>
       </c>
-      <c r="K17" s="1">
+      <c r="M17" s="1">
         <v>20</v>
       </c>
-      <c r="L17" s="1">
+      <c r="N17" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M17" s="1">
+      <c r="O17" s="1">
         <v>116168</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O17" s="1">
+      <c r="P17" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q17" s="1">
         <v>-10.2</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:17">
       <c r="A18" s="1" t="s">
         <v>91</v>
       </c>
@@ -4648,26 +4907,32 @@
       <c r="F18" s="1">
         <v>63</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J18" s="1">
+        <v>31</v>
+      </c>
+      <c r="K18" s="1">
         <v>0</v>
       </c>
-      <c r="J18" s="1">
+      <c r="L18" s="1">
         <v>3</v>
       </c>
-      <c r="K18" s="1">
+      <c r="M18" s="1">
         <v>35</v>
       </c>
-      <c r="L18" s="1">
+      <c r="N18" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M18" s="1">
+      <c r="O18" s="1">
         <v>116168</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15">
+      <c r="P18" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="1" t="s">
         <v>92</v>
       </c>
@@ -4692,29 +4957,35 @@
       <c r="H19" s="1">
         <v>36601.6</v>
       </c>
-      <c r="I19" s="1">
+      <c r="I19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J19" s="1">
+        <v>13</v>
+      </c>
+      <c r="K19" s="1">
         <v>0.06</v>
       </c>
-      <c r="J19" s="1">
+      <c r="L19" s="1">
         <v>1</v>
       </c>
-      <c r="K19" s="1">
+      <c r="M19" s="1">
         <v>32</v>
       </c>
-      <c r="L19" s="1">
+      <c r="N19" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M19" s="1">
+      <c r="O19" s="1">
         <v>116168</v>
       </c>
-      <c r="N19" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O19" s="1">
+      <c r="P19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q19" s="1">
         <v>-32.9</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:17">
       <c r="A20" s="1" t="s">
         <v>93</v>
       </c>
@@ -4739,29 +5010,35 @@
       <c r="H20" s="1">
         <v>28430.23</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J20" s="1">
+        <v>4</v>
+      </c>
+      <c r="K20" s="1">
         <v>0.15</v>
       </c>
-      <c r="J20" s="1">
+      <c r="L20" s="1">
         <v>1</v>
       </c>
-      <c r="K20" s="1">
+      <c r="M20" s="1">
         <v>29</v>
       </c>
-      <c r="L20" s="1">
+      <c r="N20" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M20" s="1">
+      <c r="O20" s="1">
         <v>112000</v>
       </c>
-      <c r="N20" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O20" s="1">
+      <c r="P20" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q20" s="1">
         <v>-28.3</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:17">
       <c r="A21" s="1" t="s">
         <v>94</v>
       </c>
@@ -4786,29 +5063,35 @@
       <c r="H21" s="1">
         <v>32030.46</v>
       </c>
-      <c r="I21" s="1">
+      <c r="I21" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J21" s="1">
+        <v>8</v>
+      </c>
+      <c r="K21" s="1">
         <v>0.52</v>
       </c>
-      <c r="J21" s="1">
+      <c r="L21" s="1">
         <v>2</v>
       </c>
-      <c r="K21" s="1">
+      <c r="M21" s="1">
         <v>17</v>
       </c>
-      <c r="L21" s="1">
+      <c r="N21" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M21" s="1">
+      <c r="O21" s="1">
         <v>112000</v>
       </c>
-      <c r="N21" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O21" s="1">
+      <c r="P21" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q21" s="1">
         <v>-7.4</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:17">
       <c r="A22" s="1" t="s">
         <v>95</v>
       </c>
@@ -4833,29 +5116,35 @@
       <c r="H22" s="1">
         <v>37495</v>
       </c>
-      <c r="I22" s="1">
+      <c r="I22" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J22" s="1">
+        <v>3</v>
+      </c>
+      <c r="K22" s="1">
         <v>0</v>
       </c>
-      <c r="J22" s="1">
+      <c r="L22" s="1">
         <v>1</v>
       </c>
-      <c r="K22" s="1">
+      <c r="M22" s="1">
         <v>34</v>
       </c>
-      <c r="L22" s="1">
+      <c r="N22" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M22" s="1">
+      <c r="O22" s="1">
         <v>84990</v>
       </c>
-      <c r="N22" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O22" s="1">
+      <c r="P22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q22" s="1">
         <v>-45</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:17">
       <c r="A23" s="1" t="s">
         <v>96</v>
       </c>
@@ -4880,29 +5169,35 @@
       <c r="H23" s="1">
         <v>41845.81</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J23" s="1">
+        <v>21</v>
+      </c>
+      <c r="K23" s="1">
         <v>0.09</v>
       </c>
-      <c r="J23" s="1">
+      <c r="L23" s="1">
         <v>1</v>
       </c>
-      <c r="K23" s="1">
-        <v>31</v>
-      </c>
-      <c r="L23" s="1">
+      <c r="M23" s="1">
+        <v>31</v>
+      </c>
+      <c r="N23" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M23" s="1">
+      <c r="O23" s="1">
         <v>84990</v>
       </c>
-      <c r="N23" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O23" s="1">
+      <c r="P23" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q23" s="1">
         <v>-30.3</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:17">
       <c r="A24" s="1" t="s">
         <v>97</v>
       </c>
@@ -4918,29 +5213,35 @@
       <c r="H24" s="1">
         <v>38333</v>
       </c>
-      <c r="I24" s="1">
+      <c r="I24" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J24" s="1">
+        <v>31</v>
+      </c>
+      <c r="K24" s="1">
         <v>0.33</v>
       </c>
-      <c r="J24" s="1">
+      <c r="L24" s="1">
         <v>2</v>
       </c>
-      <c r="K24" s="1">
+      <c r="M24" s="1">
         <v>23</v>
       </c>
-      <c r="L24" s="1">
+      <c r="N24" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M24" s="1">
+      <c r="O24" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N24" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O24" s="1">
+      <c r="P24" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q24" s="1">
         <v>-15.7</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:17">
       <c r="A25" s="1" t="s">
         <v>98</v>
       </c>
@@ -4956,29 +5257,35 @@
       <c r="H25" s="1">
         <v>33749.75</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J25" s="1">
+        <v>31</v>
+      </c>
+      <c r="K25" s="1">
         <v>0.7</v>
       </c>
-      <c r="J25" s="1">
+      <c r="L25" s="1">
         <v>3</v>
       </c>
-      <c r="K25" s="1">
+      <c r="M25" s="1">
         <v>11</v>
       </c>
-      <c r="L25" s="1">
+      <c r="N25" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M25" s="1">
+      <c r="O25" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N25" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O25" s="1">
+      <c r="P25" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q25" s="1">
         <v>-1</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:17">
       <c r="A26" s="1" t="s">
         <v>99</v>
       </c>
@@ -4994,29 +5301,35 @@
       <c r="H26" s="1">
         <v>38749.75</v>
       </c>
-      <c r="I26" s="1">
+      <c r="I26" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J26" s="1">
+        <v>31</v>
+      </c>
+      <c r="K26" s="1">
         <v>0.88</v>
       </c>
-      <c r="J26" s="1">
+      <c r="L26" s="1">
         <v>4</v>
       </c>
-      <c r="K26" s="1">
+      <c r="M26" s="1">
         <v>5</v>
       </c>
-      <c r="L26" s="1">
+      <c r="N26" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M26" s="1">
+      <c r="O26" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N26" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O26" s="1">
+      <c r="P26" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q26" s="1">
         <v>13.7</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:17">
       <c r="A27" s="1" t="s">
         <v>100</v>
       </c>
@@ -5032,29 +5345,35 @@
       <c r="H27" s="1">
         <v>32075.28</v>
       </c>
-      <c r="I27" s="1">
+      <c r="I27" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J27" s="1">
+        <v>31</v>
+      </c>
+      <c r="K27" s="1">
         <v>0.9399999999999999</v>
       </c>
-      <c r="J27" s="1">
+      <c r="L27" s="1">
         <v>4</v>
       </c>
-      <c r="K27" s="1">
+      <c r="M27" s="1">
         <v>3</v>
       </c>
-      <c r="L27" s="1">
+      <c r="N27" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M27" s="1">
+      <c r="O27" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N27" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O27" s="1">
+      <c r="P27" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q27" s="1">
         <v>24.7</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:17">
       <c r="A28" s="1" t="s">
         <v>101</v>
       </c>
@@ -5079,29 +5398,35 @@
       <c r="H28" s="1">
         <v>42499.5</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J28" s="1">
+        <v>11</v>
+      </c>
+      <c r="K28" s="1">
         <v>0.03</v>
       </c>
-      <c r="J28" s="1">
+      <c r="L28" s="1">
         <v>1</v>
       </c>
-      <c r="K28" s="1">
+      <c r="M28" s="1">
         <v>33</v>
       </c>
-      <c r="L28" s="1">
+      <c r="N28" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M28" s="1">
+      <c r="O28" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N28" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O28" s="1">
+      <c r="P28" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q28" s="1">
         <v>-37.7</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:17">
       <c r="A29" s="1" t="s">
         <v>102</v>
       </c>
@@ -5117,26 +5442,32 @@
       <c r="F29" s="1">
         <v>115</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J29" s="1">
+        <v>31</v>
+      </c>
+      <c r="K29" s="1">
         <v>0</v>
       </c>
-      <c r="J29" s="1">
+      <c r="L29" s="1">
         <v>4</v>
       </c>
-      <c r="K29" s="1">
+      <c r="M29" s="1">
         <v>35</v>
       </c>
-      <c r="L29" s="1">
+      <c r="N29" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M29" s="1">
+      <c r="O29" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N29" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15">
+      <c r="P29" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" s="1" t="s">
         <v>103</v>
       </c>
@@ -5152,26 +5483,32 @@
       <c r="F30" s="1">
         <v>123</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J30" s="1">
+        <v>31</v>
+      </c>
+      <c r="K30" s="1">
         <v>0</v>
       </c>
-      <c r="J30" s="1">
+      <c r="L30" s="1">
         <v>4</v>
       </c>
-      <c r="K30" s="1">
+      <c r="M30" s="1">
         <v>35</v>
       </c>
-      <c r="L30" s="1">
+      <c r="N30" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M30" s="1">
+      <c r="O30" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N30" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15">
+      <c r="P30" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" s="1" t="s">
         <v>104</v>
       </c>
@@ -5196,29 +5533,35 @@
       <c r="H31" s="1">
         <v>30249.75</v>
       </c>
-      <c r="I31" s="1">
-        <v>0.36</v>
+      <c r="I31" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="J31" s="1">
         <v>2</v>
       </c>
       <c r="K31" s="1">
+        <v>0.36</v>
+      </c>
+      <c r="L31" s="1">
+        <v>2</v>
+      </c>
+      <c r="M31" s="1">
         <v>22</v>
       </c>
-      <c r="L31" s="1">
+      <c r="N31" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M31" s="1">
+      <c r="O31" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N31" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O31" s="1">
+      <c r="P31" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q31" s="1">
         <v>-11.3</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:17">
       <c r="A32" s="1" t="s">
         <v>105</v>
       </c>
@@ -5243,29 +5586,35 @@
       <c r="H32" s="1">
         <v>24999.81</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J32" s="1">
+        <v>1</v>
+      </c>
+      <c r="K32" s="1">
         <v>0.58</v>
       </c>
-      <c r="J32" s="1">
+      <c r="L32" s="1">
         <v>3</v>
       </c>
-      <c r="K32" s="1">
+      <c r="M32" s="1">
         <v>15</v>
       </c>
-      <c r="L32" s="1">
+      <c r="N32" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M32" s="1">
+      <c r="O32" s="1">
         <v>130141.86</v>
       </c>
-      <c r="N32" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O32" s="1">
+      <c r="P32" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q32" s="1">
         <v>-4.7</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:17">
       <c r="A33" s="1" t="s">
         <v>106</v>
       </c>
@@ -5290,29 +5639,35 @@
       <c r="H33" s="1">
         <v>42592.59</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J33" s="1">
+        <v>22</v>
+      </c>
+      <c r="K33" s="1">
         <v>0.76</v>
       </c>
-      <c r="J33" s="1">
+      <c r="L33" s="1">
         <v>3</v>
       </c>
-      <c r="K33" s="1">
+      <c r="M33" s="1">
         <v>9</v>
       </c>
-      <c r="L33" s="1">
+      <c r="N33" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M33" s="1">
+      <c r="O33" s="1">
         <v>131499.5</v>
       </c>
-      <c r="N33" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O33" s="1">
+      <c r="P33" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q33" s="1">
         <v>1.2</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:17">
       <c r="A34" s="1" t="s">
         <v>107</v>
       </c>
@@ -5337,29 +5692,35 @@
       <c r="H34" s="1">
         <v>38579.94</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J34" s="1">
+        <v>15</v>
+      </c>
+      <c r="K34" s="1">
         <v>0.45</v>
       </c>
-      <c r="J34" s="1">
+      <c r="L34" s="1">
         <v>2</v>
       </c>
-      <c r="K34" s="1">
+      <c r="M34" s="1">
         <v>19</v>
       </c>
-      <c r="L34" s="1">
+      <c r="N34" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M34" s="1">
+      <c r="O34" s="1">
         <v>131499.5</v>
       </c>
-      <c r="N34" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O34" s="1">
+      <c r="P34" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q34" s="1">
         <v>-8.300000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:17">
       <c r="A35" s="1" t="s">
         <v>108</v>
       </c>
@@ -5384,29 +5745,35 @@
       <c r="H35" s="1">
         <v>37972.7</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" s="1">
+        <v>23</v>
+      </c>
+      <c r="K35" s="1">
         <v>0.79</v>
       </c>
-      <c r="J35" s="1">
+      <c r="L35" s="1">
         <v>4</v>
       </c>
-      <c r="K35" s="1">
+      <c r="M35" s="1">
         <v>8</v>
       </c>
-      <c r="L35" s="1">
+      <c r="N35" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M35" s="1">
+      <c r="O35" s="1">
         <v>153249.5</v>
       </c>
-      <c r="N35" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O35" s="1">
+      <c r="P35" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q35" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:17">
       <c r="A36" s="1" t="s">
         <v>109</v>
       </c>
@@ -5431,29 +5798,35 @@
       <c r="H36" s="1">
         <v>33200</v>
       </c>
-      <c r="I36" s="1">
+      <c r="I36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J36" s="1">
+        <v>9</v>
+      </c>
+      <c r="K36" s="1">
         <v>0.91</v>
       </c>
-      <c r="J36" s="1">
+      <c r="L36" s="1">
         <v>4</v>
       </c>
-      <c r="K36" s="1">
+      <c r="M36" s="1">
         <v>4</v>
       </c>
-      <c r="L36" s="1">
+      <c r="N36" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M36" s="1">
+      <c r="O36" s="1">
         <v>153249.5</v>
       </c>
-      <c r="N36" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O36" s="1">
+      <c r="P36" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q36" s="1">
         <v>21.7</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:17">
       <c r="A37" s="1" t="s">
         <v>110</v>
       </c>
@@ -5478,29 +5851,35 @@
       <c r="H37" s="1">
         <v>41358.26</v>
       </c>
-      <c r="I37" s="1">
+      <c r="I37" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J37" s="1">
+        <v>16</v>
+      </c>
+      <c r="K37" s="1">
         <v>0.12</v>
       </c>
-      <c r="J37" s="1">
+      <c r="L37" s="1">
         <v>1</v>
       </c>
-      <c r="K37" s="1">
+      <c r="M37" s="1">
         <v>30</v>
       </c>
-      <c r="L37" s="1">
+      <c r="N37" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M37" s="1">
+      <c r="O37" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N37" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O37" s="1">
+      <c r="P37" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q37" s="1">
         <v>-30.2</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:17">
       <c r="A38" s="1" t="s">
         <v>111</v>
       </c>
@@ -5525,29 +5904,35 @@
       <c r="H38" s="1">
         <v>33858.71</v>
       </c>
-      <c r="I38" s="1">
+      <c r="I38" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J38" s="1">
+        <v>17</v>
+      </c>
+      <c r="K38" s="1">
         <v>0.18</v>
       </c>
-      <c r="J38" s="1">
+      <c r="L38" s="1">
         <v>1</v>
       </c>
-      <c r="K38" s="1">
+      <c r="M38" s="1">
         <v>28</v>
       </c>
-      <c r="L38" s="1">
+      <c r="N38" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M38" s="1">
+      <c r="O38" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N38" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O38" s="1">
+      <c r="P38" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q38" s="1">
         <v>-23</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:17">
       <c r="A39" s="1" t="s">
         <v>112</v>
       </c>
@@ -5572,29 +5957,35 @@
       <c r="H39" s="1">
         <v>31485.71</v>
       </c>
-      <c r="I39" s="1">
+      <c r="I39" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J39" s="1">
+        <v>7</v>
+      </c>
+      <c r="K39" s="1">
         <v>0.27</v>
       </c>
-      <c r="J39" s="1">
+      <c r="L39" s="1">
         <v>2</v>
       </c>
-      <c r="K39" s="1">
+      <c r="M39" s="1">
         <v>25</v>
       </c>
-      <c r="L39" s="1">
+      <c r="N39" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M39" s="1">
+      <c r="O39" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N39" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O39" s="1">
+      <c r="P39" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q39" s="1">
         <v>-19.2</v>
       </c>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" spans="1:17">
       <c r="A40" s="1" t="s">
         <v>113</v>
       </c>
@@ -5619,29 +6010,35 @@
       <c r="H40" s="1">
         <v>32500.29</v>
       </c>
-      <c r="I40" s="1">
+      <c r="I40" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J40" s="1">
+        <v>10</v>
+      </c>
+      <c r="K40" s="1">
         <v>0.3</v>
       </c>
-      <c r="J40" s="1">
+      <c r="L40" s="1">
         <v>2</v>
       </c>
-      <c r="K40" s="1">
+      <c r="M40" s="1">
         <v>24</v>
       </c>
-      <c r="L40" s="1">
+      <c r="N40" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M40" s="1">
+      <c r="O40" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N40" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O40" s="1">
+      <c r="P40" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q40" s="1">
         <v>-16.6</v>
       </c>
     </row>
-    <row r="41" spans="1:15">
+    <row r="41" spans="1:17">
       <c r="A41" s="1" t="s">
         <v>114</v>
       </c>
@@ -5666,29 +6063,35 @@
       <c r="H41" s="1">
         <v>27731.91</v>
       </c>
-      <c r="I41" s="1">
+      <c r="I41" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J41" s="1">
+        <v>6</v>
+      </c>
+      <c r="K41" s="1">
         <v>0.61</v>
       </c>
-      <c r="J41" s="1">
+      <c r="L41" s="1">
         <v>3</v>
       </c>
-      <c r="K41" s="1">
+      <c r="M41" s="1">
         <v>14</v>
       </c>
-      <c r="L41" s="1">
+      <c r="N41" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M41" s="1">
+      <c r="O41" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N41" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="O41" s="1">
+      <c r="P41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q41" s="1">
         <v>-4.4</v>
       </c>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" spans="1:17">
       <c r="A42" s="1" t="s">
         <v>115</v>
       </c>
@@ -5713,29 +6116,35 @@
       <c r="H42" s="1">
         <v>27712.64</v>
       </c>
-      <c r="I42" s="1">
+      <c r="I42" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J42" s="1">
+        <v>5</v>
+      </c>
+      <c r="K42" s="1">
         <v>0.82</v>
       </c>
-      <c r="J42" s="1">
+      <c r="L42" s="1">
         <v>4</v>
       </c>
-      <c r="K42" s="1">
+      <c r="M42" s="1">
         <v>7</v>
       </c>
-      <c r="L42" s="1">
+      <c r="N42" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M42" s="1">
+      <c r="O42" s="1">
         <v>116875.67</v>
       </c>
-      <c r="N42" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O42" s="1">
+      <c r="P42" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q42" s="1">
         <v>7.7</v>
       </c>
     </row>
-    <row r="43" spans="1:15">
+    <row r="43" spans="1:17">
       <c r="A43" s="1" t="s">
         <v>116</v>
       </c>
@@ -5760,29 +6169,35 @@
       <c r="H43" s="1">
         <v>42112.68</v>
       </c>
-      <c r="I43" s="1">
+      <c r="I43" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J43" s="1">
+        <v>30</v>
+      </c>
+      <c r="K43" s="1">
         <v>0.97</v>
       </c>
-      <c r="J43" s="1">
+      <c r="L43" s="1">
         <v>4</v>
       </c>
-      <c r="K43" s="1">
+      <c r="M43" s="1">
         <v>2</v>
       </c>
-      <c r="L43" s="1">
+      <c r="N43" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M43" s="1">
+      <c r="O43" s="1">
         <v>349000</v>
       </c>
-      <c r="N43" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O43" s="1">
+      <c r="P43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q43" s="1">
         <v>119.3</v>
       </c>
     </row>
-    <row r="44" spans="1:15">
+    <row r="44" spans="1:17">
       <c r="A44" s="1" t="s">
         <v>117</v>
       </c>
@@ -5807,25 +6222,31 @@
       <c r="H44" s="1">
         <v>38737.86</v>
       </c>
-      <c r="I44" s="1">
-        <v>1</v>
+      <c r="I44" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="J44" s="1">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="K44" s="1">
         <v>1</v>
       </c>
       <c r="L44" s="1">
+        <v>4</v>
+      </c>
+      <c r="M44" s="1">
+        <v>1</v>
+      </c>
+      <c r="N44" s="1">
         <v>136349.21</v>
       </c>
-      <c r="M44" s="1">
+      <c r="O44" s="1">
         <v>349000</v>
       </c>
-      <c r="N44" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O44" s="1">
+      <c r="P44" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q44" s="1">
         <v>192.6</v>
       </c>
     </row>
@@ -5860,7 +6281,7 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -5868,7 +6289,7 @@
         <v>48</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>51</v>
@@ -5883,37 +6304,37 @@
         <v>124</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>4</v>
@@ -5939,19 +6360,19 @@
         <v>93</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L3" s="1">
         <v>1</v>
@@ -5995,19 +6416,19 @@
         <v>93</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L4" s="1">
         <v>2</v>
@@ -6045,19 +6466,19 @@
         <v>3.7</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L5" s="1">
         <v>5</v>
@@ -6095,19 +6516,19 @@
         <v>3.7</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L6" s="1">
         <v>6</v>
@@ -6145,19 +6566,19 @@
         <v>2.9</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L7" s="1">
         <v>7</v>
@@ -6195,19 +6616,19 @@
         <v>3.7</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L8" s="1">
         <v>8</v>
@@ -6248,19 +6669,19 @@
         <v>2.9</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L9" s="1">
         <v>1</v>
@@ -6301,19 +6722,19 @@
         <v>3.7</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L10" s="1">
         <v>3</v>
@@ -6354,19 +6775,19 @@
         <v>2.9</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L11" s="1">
         <v>2</v>
@@ -6407,19 +6828,19 @@
         <v>3.7</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L12" s="1">
         <v>4</v>
@@ -6463,19 +6884,19 @@
         <v>60</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L13" s="1">
         <v>2</v>
@@ -6519,19 +6940,19 @@
         <v>75</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L14" s="1">
         <v>1</v>
@@ -6572,19 +6993,19 @@
         <v>63</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L15" s="1">
         <v>4</v>
@@ -6628,19 +7049,19 @@
         <v>73</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L16" s="1">
         <v>3</v>
@@ -6684,19 +7105,19 @@
         <v>73</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L17" s="1">
         <v>2</v>
@@ -6737,19 +7158,19 @@
         <v>63</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L18" s="1">
         <v>5</v>
@@ -6793,19 +7214,19 @@
         <v>55</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L19" s="1">
         <v>1</v>
@@ -6849,19 +7270,19 @@
         <v>80</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L20" s="1">
         <v>1</v>
@@ -6905,19 +7326,19 @@
         <v>80</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L21" s="1">
         <v>2</v>
@@ -6961,19 +7382,19 @@
         <v>50</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L22" s="1">
         <v>1</v>
@@ -7017,19 +7438,19 @@
         <v>60</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L23" s="1">
         <v>2</v>
@@ -7067,19 +7488,19 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L24" s="1">
         <v>2</v>
@@ -7117,19 +7538,19 @@
         <v>4</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L25" s="1">
         <v>5</v>
@@ -7167,19 +7588,19 @@
         <v>4</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L26" s="1">
         <v>6</v>
@@ -7217,19 +7638,19 @@
         <v>5.3</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L27" s="1">
         <v>7</v>
@@ -7273,19 +7694,19 @@
         <v>101</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L28" s="1">
         <v>1</v>
@@ -7326,19 +7747,19 @@
         <v>115</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L29" s="1">
         <v>8</v>
@@ -7379,19 +7800,19 @@
         <v>123</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L30" s="1">
         <v>9</v>
@@ -7435,19 +7856,19 @@
         <v>125</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L31" s="1">
         <v>3</v>
@@ -7491,19 +7912,19 @@
         <v>125</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L32" s="1">
         <v>4</v>
@@ -7547,19 +7968,19 @@
         <v>85</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L33" s="1">
         <v>2</v>
@@ -7603,19 +8024,19 @@
         <v>85</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L34" s="1">
         <v>1</v>
@@ -7659,19 +8080,19 @@
         <v>105</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L35" s="1">
         <v>1</v>
@@ -7715,19 +8136,19 @@
         <v>105</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L36" s="1">
         <v>2</v>
@@ -7771,19 +8192,19 @@
         <v>68</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L37" s="1">
         <v>1</v>
@@ -7827,19 +8248,19 @@
         <v>82</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L38" s="1">
         <v>2</v>
@@ -7883,19 +8304,19 @@
         <v>82</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L39" s="1">
         <v>3</v>
@@ -7939,19 +8360,19 @@
         <v>82</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L40" s="1">
         <v>4</v>
@@ -7995,19 +8416,19 @@
         <v>82</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L41" s="1">
         <v>5</v>
@@ -8051,19 +8472,19 @@
         <v>82</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L42" s="1">
         <v>6</v>
@@ -8107,19 +8528,19 @@
         <v>155</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="L43" s="1">
         <v>1</v>
@@ -8163,19 +8584,19 @@
         <v>155</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="L44" s="1">
         <v>2</v>
@@ -8215,127 +8636,127 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -8345,7 +8766,446 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="45.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="45.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C3" s="1">
+        <v>41000</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F3" s="1">
+        <v>184.5</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2022</v>
+      </c>
+      <c r="C4" s="1">
+        <v>249000</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E4" s="1">
+        <v>507.3</v>
+      </c>
+      <c r="F4" s="1">
+        <v>184.5</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2023</v>
+      </c>
+      <c r="C5" s="1">
+        <v>728000</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="1">
+        <v>192.4</v>
+      </c>
+      <c r="F5" s="1">
+        <v>184.5</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C6" s="1">
+        <v>944000</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E6" s="1">
+        <v>29.7</v>
+      </c>
+      <c r="F6" s="1">
+        <v>184.5</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="25.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="26.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="41.7109375" style="1" customWidth="1"/>
+    <col min="17" max="18" width="27.7109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="23.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19">
+      <c r="A1" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="A2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="1">
+        <v>944000</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="1">
+        <v>10</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1038400</v>
+      </c>
+      <c r="G3" s="1">
+        <v>12460.8</v>
+      </c>
+      <c r="H3" s="1">
+        <v>60</v>
+      </c>
+      <c r="I3" s="1">
+        <v>70</v>
+      </c>
+      <c r="J3" s="1">
+        <v>436128</v>
+      </c>
+      <c r="K3" s="1">
+        <v>5233.5</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="M3" s="1">
+        <v>6541</v>
+      </c>
+      <c r="N3" s="1">
+        <v>78.5</v>
+      </c>
+      <c r="O3" s="1">
+        <v>120000</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="1">
+        <v>944000</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E4" s="1">
+        <v>25</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1180000</v>
+      </c>
+      <c r="G4" s="1">
+        <v>14687</v>
+      </c>
+      <c r="H4" s="1">
+        <v>70</v>
+      </c>
+      <c r="I4" s="1">
+        <v>80</v>
+      </c>
+      <c r="J4" s="1">
+        <v>660800</v>
+      </c>
+      <c r="K4" s="1">
+        <v>8224.700000000001</v>
+      </c>
+      <c r="L4" s="1">
+        <v>3</v>
+      </c>
+      <c r="M4" s="1">
+        <v>19824</v>
+      </c>
+      <c r="N4" s="1">
+        <v>246.7</v>
+      </c>
+      <c r="O4" s="1">
+        <v>124466</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C5" s="1">
+        <v>944000</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E5" s="1">
+        <v>45</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1368800</v>
+      </c>
+      <c r="G5" s="1">
+        <v>17794.4</v>
+      </c>
+      <c r="H5" s="1">
+        <v>80</v>
+      </c>
+      <c r="I5" s="1">
+        <v>85</v>
+      </c>
+      <c r="J5" s="1">
+        <v>930784</v>
+      </c>
+      <c r="K5" s="1">
+        <v>12100.2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>5</v>
+      </c>
+      <c r="M5" s="1">
+        <v>46539</v>
+      </c>
+      <c r="N5" s="1">
+        <v>605</v>
+      </c>
+      <c r="O5" s="1">
+        <v>130000</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.7109375" style="1" customWidth="1"/>
@@ -8353,7 +9213,8 @@
     <col min="5" max="5" width="15.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="16.7109375" style="1" customWidth="1"/>
-    <col min="8" max="9" width="17.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" style="1" customWidth="1"/>
     <col min="10" max="11" width="26.7109375" style="1" customWidth="1"/>
     <col min="12" max="12" width="33.7109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="41.7109375" style="1" customWidth="1"/>
@@ -8363,274 +9224,274 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="2" t="s">
-        <v>279</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="3" t="s">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>210</v>
+        <v>257</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>211</v>
+        <v>258</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>212</v>
+        <v>259</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>213</v>
+        <v>260</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>214</v>
+        <v>261</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>215</v>
+        <v>262</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>216</v>
+        <v>263</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>218</v>
+        <v>265</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>219</v>
+        <v>266</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>220</v>
+        <v>267</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>221</v>
+        <v>268</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>222</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="1" t="s">
-        <v>223</v>
+        <v>270</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>228</v>
+        <v>276</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>234</v>
+        <v>283</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>240</v>
+        <v>290</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>255</v>
+        <v>307</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>263</v>
+        <v>316</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>267</v>
+        <v>320</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>273</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1" t="s">
-        <v>224</v>
+        <v>271</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>229</v>
+        <v>277</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>235</v>
+        <v>284</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>240</v>
+        <v>290</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>246</v>
+        <v>297</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>250</v>
+        <v>301</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>256</v>
+        <v>308</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>263</v>
+        <v>316</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>267</v>
+        <v>320</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>274</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1" t="s">
-        <v>225</v>
+        <v>272</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>230</v>
+        <v>278</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>236</v>
+        <v>285</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>264</v>
+        <v>317</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>268</v>
+        <v>321</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>275</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1" t="s">
-        <v>226</v>
+        <v>273</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>231</v>
+        <v>279</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>237</v>
+        <v>286</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>241</v>
+        <v>291</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>254</v>
+        <v>305</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>263</v>
+        <v>316</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>267</v>
+        <v>320</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>276</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1" t="s">
-        <v>227</v>
+        <v>274</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>232</v>
+        <v>280</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>238</v>
+        <v>287</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>242</v>
+        <v>292</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>247</v>
+        <v>298</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>259</v>
+        <v>311</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>261</v>
+        <v>314</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>265</v>
+        <v>318</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>269</v>
+        <v>322</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>277</v>
+        <v>329</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -8638,46 +9499,93 @@
         <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>233</v>
+        <v>281</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>239</v>
+        <v>288</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>243</v>
+        <v>293</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>248</v>
+        <v>299</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>261</v>
+        <v>314</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>31</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>266</v>
+        <v>319</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>270</v>
+        <v>224</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>278</v>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -8686,12 +9594,13 @@
     <hyperlink ref="D4" r:id="rId2"/>
     <hyperlink ref="D6" r:id="rId3"/>
     <hyperlink ref="D7" r:id="rId4"/>
+    <hyperlink ref="D9" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8703,92 +9612,92 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>305</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>281</v>
+        <v>334</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>282</v>
+        <v>335</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>283</v>
+        <v>336</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>284</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>285</v>
+        <v>338</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>289</v>
+        <v>342</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>293</v>
+        <v>346</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>297</v>
+        <v>350</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>301</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>286</v>
+        <v>339</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>290</v>
+        <v>343</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>294</v>
+        <v>347</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>298</v>
+        <v>351</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>302</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>287</v>
+        <v>340</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>291</v>
+        <v>344</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>295</v>
+        <v>348</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>299</v>
+        <v>352</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>303</v>
+        <v>356</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>288</v>
+        <v>341</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>296</v>
+        <v>349</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>300</v>
+        <v>353</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>304</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>